<commit_message>
Corrida | ARG-MVDO | 2026-02-20 18:53:49.119075
</commit_message>
<xml_diff>
--- a/web_ces/indicadores/ARG-M_out.xlsx
+++ b/web_ces/indicadores/ARG-M_out.xlsx
@@ -2242,7 +2242,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.677674314823471</v>
+        <v>0.677889163879187</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2300,7 +2300,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.426188050814718</v>
+        <v>0.426422816200978</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2370,7 +2370,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.0171575487463079</v>
+        <v>0.0175276891424079</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2400,7 +2400,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.000000465828698461128</v>
+        <v>0.000000489723468281191</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -29679,7 +29679,7 @@
         <v>546</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.0857247726010663</v>
+        <v>0.085431019401934</v>
       </c>
     </row>
     <row r="6">
@@ -29687,7 +29687,7 @@
         <v>547</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.159492182615541</v>
+        <v>0.159673545500643</v>
       </c>
     </row>
     <row r="7">
@@ -29695,7 +29695,7 @@
         <v>548</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.261592368269234</v>
+        <v>0.262003485885144</v>
       </c>
     </row>
     <row r="8">
@@ -29703,7 +29703,7 @@
         <v>549</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.366791718681542</v>
+        <v>0.367051657091359</v>
       </c>
     </row>
     <row r="9">
@@ -29711,7 +29711,7 @@
         <v>550</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.451197959901701</v>
+        <v>0.451322333432685</v>
       </c>
     </row>
     <row r="10">
@@ -29719,7 +29719,7 @@
         <v>551</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.502295391808575</v>
+        <v>0.502423488724627</v>
       </c>
     </row>
     <row r="11">
@@ -29727,7 +29727,7 @@
         <v>552</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.541395273873647</v>
+        <v>0.541434620019055</v>
       </c>
     </row>
     <row r="12">
@@ -29735,7 +29735,7 @@
         <v>553</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.587435295909586</v>
+        <v>0.587439391797211</v>
       </c>
     </row>
     <row r="13">
@@ -29743,7 +29743,7 @@
         <v>554</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.626033180791381</v>
+        <v>0.626051953853543</v>
       </c>
     </row>
     <row r="14">
@@ -29751,7 +29751,7 @@
         <v>555</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.65283079799801</v>
+        <v>0.653010578934966</v>
       </c>
     </row>
     <row r="15">
@@ -29759,7 +29759,7 @@
         <v>556</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.677674314823471</v>
+        <v>0.677889163879187</v>
       </c>
     </row>
     <row r="16">
@@ -29767,7 +29767,7 @@
         <v>557</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.646692657425427</v>
+        <v>0.646745143720181</v>
       </c>
     </row>
     <row r="17">
@@ -29775,7 +29775,7 @@
         <v>558</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.554856215628535</v>
+        <v>0.554968277097625</v>
       </c>
     </row>
     <row r="18">
@@ -29783,7 +29783,7 @@
         <v>559</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.440001222493222</v>
+        <v>0.440524185459776</v>
       </c>
     </row>
     <row r="19">
@@ -29791,7 +29791,7 @@
         <v>560</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.31627641300898</v>
+        <v>0.317139488799654</v>
       </c>
     </row>
     <row r="20">
@@ -29799,7 +29799,7 @@
         <v>561</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.208493992742397</v>
+        <v>0.209298073757197</v>
       </c>
     </row>
     <row r="21">
@@ -29807,7 +29807,7 @@
         <v>562</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.126326543492979</v>
+        <v>0.126616414982421</v>
       </c>
     </row>
     <row r="22">
@@ -29815,7 +29815,7 @@
         <v>563</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.0530387146737629</v>
+        <v>0.0528121603784903</v>
       </c>
     </row>
     <row r="23">
@@ -29823,7 +29823,7 @@
         <v>564</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.00340709004375087</v>
+        <v>-0.00371912355474429</v>
       </c>
     </row>
     <row r="24">
@@ -30066,22 +30066,22 @@
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5DA9A6F6-0984-4FB5-AD13-8964EB4DB40F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C71FB331-7D3C-45C5-9C17-DFA885454FCF}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1B42119A-EFAD-41D9-A874-E5DF9526F546}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6F68A95-8D76-48FC-90D6-BE95E5418DE8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9DE64A71-7AF4-40E5-9220-6F0F6B928F23}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{25395EC6-403A-4195-B326-00AA6AFFAF31}"/>
 </file>
</xml_diff>